<commit_message>
+ Data for Kill/Razesanity
</commit_message>
<xml_diff>
--- a/docs/Logic Requirements/Ageipelago Genghis Khan.xlsx
+++ b/docs/Logic Requirements/Ageipelago Genghis Khan.xlsx
@@ -5,15 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/BB6DD295C338E39F/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefb\OneDrive\Desktop\Logic Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="8_{36B768C8-52B4-40AF-A7C8-D3CFEFD0AF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{431BC05F-6B1D-4A6A-B318-5B28BCA61ECE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE07A875-7858-4D90-98E6-D7911BA92ACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A331DE4D-6B47-4A46-A574-F0C6C77C75AD}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{A331DE4D-6B47-4A46-A574-F0C6C77C75AD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Genghis Khan" sheetId="1" r:id="rId1"/>
+    <sheet name="Crucible" sheetId="5" r:id="rId2"/>
+    <sheet name="A Live of Revenge" sheetId="2" r:id="rId3"/>
+    <sheet name="Into China" sheetId="3" r:id="rId4"/>
+    <sheet name="The Horde Rides West" sheetId="4" r:id="rId5"/>
+    <sheet name="The Promise" sheetId="6" r:id="rId6"/>
+    <sheet name="Pax Mongolica" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="196">
   <si>
     <t>Scenario</t>
   </si>
@@ -2381,105 +2387,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Starting Units:
-2 Light Cavalry
-3 Knights
-3 Camel Riders
-8 War Elephants
-4 Crossbowmen
-10 Heavy Cavalry Archers
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Moderate:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-8 Savars
-2 Light Cavalry
-8 Elite War Elephants
-8 Heavy Cavalry Archers
-1 Trebuchet
-1 Monk
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Standard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-8 Savars
-2 Light Cavalry
-8 Elite War Elephants
-8 Heavy Cavalry Archers
-1 Scorpion
-1 Monk
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Hard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-11 Savars
-2 Light Cavalry
-11 Elite War Elephants
-10 Heavy Cavalry Archers
-3 Scorpion
-2 Trebuchets
-2 Monks</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <t xml:space="preserve">Defeating </t>
     </r>
     <r>
@@ -3001,12 +2908,559 @@
 4 Capped Rams</t>
     </r>
   </si>
+  <si>
+    <t>Killable Units</t>
+  </si>
+  <si>
+    <t>Destructible Buildings</t>
+  </si>
+  <si>
+    <t>Deer</t>
+  </si>
+  <si>
+    <t>No items required</t>
+  </si>
+  <si>
+    <t>Palisade Wall</t>
+  </si>
+  <si>
+    <t>Grey Wolf</t>
+  </si>
+  <si>
+    <t>Man-at-Arms</t>
+  </si>
+  <si>
+    <t>Archery Range</t>
+  </si>
+  <si>
+    <t>Crossbowman</t>
+  </si>
+  <si>
+    <t>Watch Tower</t>
+  </si>
+  <si>
+    <t>Scout Cavalry</t>
+  </si>
+  <si>
+    <t>Lumber Camp</t>
+  </si>
+  <si>
+    <t>Archer</t>
+  </si>
+  <si>
+    <t>Mill</t>
+  </si>
+  <si>
+    <t>Light Cavalry</t>
+  </si>
+  <si>
+    <t>House</t>
+  </si>
+  <si>
+    <t>Siege Workshop</t>
+  </si>
+  <si>
+    <t>Barracks</t>
+  </si>
+  <si>
+    <t>Stable</t>
+  </si>
+  <si>
+    <t>Capped Ram</t>
+  </si>
+  <si>
+    <t>Monastery</t>
+  </si>
+  <si>
+    <t>War Galley</t>
+  </si>
+  <si>
+    <t>Market</t>
+  </si>
+  <si>
+    <t>Trebuchet</t>
+  </si>
+  <si>
+    <t>Dock</t>
+  </si>
+  <si>
+    <t>Knight</t>
+  </si>
+  <si>
+    <t>Outpost</t>
+  </si>
+  <si>
+    <t>Monk</t>
+  </si>
+  <si>
+    <t>Guard Tower</t>
+  </si>
+  <si>
+    <t>Militia</t>
+  </si>
+  <si>
+    <t>Stone Wall</t>
+  </si>
+  <si>
+    <t>Scorpion</t>
+  </si>
+  <si>
+    <t>Stone Gate</t>
+  </si>
+  <si>
+    <t>Castle</t>
+  </si>
+  <si>
+    <t>Keep</t>
+  </si>
+  <si>
+    <t>Fortified Wall</t>
+  </si>
+  <si>
+    <t>Dire Wolf</t>
+  </si>
+  <si>
+    <t>Sheep</t>
+  </si>
+  <si>
+    <t>Ornlu the Wolf</t>
+  </si>
+  <si>
+    <t>Elite Mangudai</t>
+  </si>
+  <si>
+    <t>Genghis Khan</t>
+  </si>
+  <si>
+    <t>No items required
+Disappears after Intro</t>
+  </si>
+  <si>
+    <t>Cavalry Archer</t>
+  </si>
+  <si>
+    <t>Rocket Cart</t>
+  </si>
+  <si>
+    <t>Mangudai</t>
+  </si>
+  <si>
+    <t>Camel Rider</t>
+  </si>
+  <si>
+    <t>Yurt</t>
+  </si>
+  <si>
+    <t>Yurt (Large)</t>
+  </si>
+  <si>
+    <t>Villager</t>
+  </si>
+  <si>
+    <t>Skirmisher</t>
+  </si>
+  <si>
+    <t>Elite Skirmisher</t>
+  </si>
+  <si>
+    <t>Kushluk</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Mangudai
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <t>Mining Camp</t>
+  </si>
+  <si>
+    <t>Town Center</t>
+  </si>
+  <si>
+    <t>Blacksmith</t>
+  </si>
+  <si>
+    <t>Pasture</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Castle
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <t>Wild Boar</t>
+  </si>
+  <si>
+    <t>Fire Lancer</t>
+  </si>
+  <si>
+    <t>Heavy Rocket Cart</t>
+  </si>
+  <si>
+    <t>Battering Ram</t>
+  </si>
+  <si>
+    <t>Siege Ram</t>
+  </si>
+  <si>
+    <t>Heavy Scorpion</t>
+  </si>
+  <si>
+    <t>Chu-Ko-Nu</t>
+  </si>
+  <si>
+    <t>Elite Chu-Ko-Nu</t>
+  </si>
+  <si>
+    <t>Galley</t>
+  </si>
+  <si>
+    <t>Galleon</t>
+  </si>
+  <si>
+    <t>Grenadier</t>
+  </si>
+  <si>
+    <t>Iron Pagoda</t>
+  </si>
+  <si>
+    <t>Elite Iron Pagoda</t>
+  </si>
+  <si>
+    <t>Steppe Lancer</t>
+  </si>
+  <si>
+    <t>Arbalester</t>
+  </si>
+  <si>
+    <t>Long Swordsman</t>
+  </si>
+  <si>
+    <t>Two-Handed Swordsman</t>
+  </si>
+  <si>
+    <t>Champion</t>
+  </si>
+  <si>
+    <t>Requires Dock</t>
+  </si>
+  <si>
+    <t>Requires Transport Ship</t>
+  </si>
+  <si>
+    <t>Farm</t>
+  </si>
+  <si>
+    <t>Fence</t>
+  </si>
+  <si>
+    <t>University</t>
+  </si>
+  <si>
+    <t>Wonder</t>
+  </si>
+  <si>
+    <t>Bear</t>
+  </si>
+  <si>
+    <t>Boyar</t>
+  </si>
+  <si>
+    <t>Heavy Cavalry Archer</t>
+  </si>
+  <si>
+    <t>War Elephant</t>
+  </si>
+  <si>
+    <t>Elite War Elephant</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Starting Units:
+2 Light Cavalry
+3 Knights
+3 Camel Riders
+8 War Elephants
+4 Crossbowmen
+10 Heavy Cavalry Archers
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moderate:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+8 Savars
+2 Light Cavalry
+8 Elite War Elephants
+8 Heavy Cavalry Archers
+1 Trebuchet
+1 Monk
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Standard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+8 Savars
+2 Light Cavalry
+8 Elite War Elephants
+8 Heavy Cavalry Archers
+1 Scorpion
+1 Monk
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+11 Savars
+2 Light Cavalry
+11 Elite War Elephants
+10 Heavy Cavalry Archers
+3 Scorpions
+2 Trebuchets
+2 Monks</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Scorpion
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Not on Moderate)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Trebuchet
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Trade Workshop</t>
+  </si>
+  <si>
+    <t>Mangonel</t>
+  </si>
+  <si>
+    <t>Cavalier</t>
+  </si>
+  <si>
+    <t>Pikeman</t>
+  </si>
+  <si>
+    <t>Halberdier</t>
+  </si>
+  <si>
+    <t>Teutonic Knight</t>
+  </si>
+  <si>
+    <t>Elite Teutonic Knight</t>
+  </si>
+  <si>
+    <t>Paladin</t>
+  </si>
+  <si>
+    <t>Siege Onager</t>
+  </si>
+  <si>
+    <t>Folwark</t>
+  </si>
+  <si>
+    <t>City Wall</t>
+  </si>
+  <si>
+    <t>Bombard Tower</t>
+  </si>
+  <si>
+    <t>Fortified Gate</t>
+  </si>
+  <si>
+    <t>Pavilion</t>
+  </si>
+  <si>
+    <t>Pavilion (Large)</t>
+  </si>
+  <si>
+    <t>Magyar Huszar</t>
+  </si>
+  <si>
+    <t>Elite Magyar Huszar</t>
+  </si>
+  <si>
+    <t>Hussar</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Elite Fire Lancer</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Mounted Trebuchet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Onager</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(not on Standard)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3157,16 +3611,88 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFFC000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF30F2FC"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -3254,11 +3780,96 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3294,6 +3905,177 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3851,14 +4633,14 @@
         <v>77</v>
       </c>
       <c r="L7" s="8" t="s">
-        <v>78</v>
+        <v>171</v>
       </c>
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="2:17" ht="394.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -3883,20 +4665,20 @@
       </c>
       <c r="I8" s="11"/>
       <c r="J8" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="L8" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="K8" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="L8" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="M8" s="8"/>
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
@@ -3923,7 +4705,7 @@
         <v>47</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8"/>
@@ -3937,4 +4719,2569 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31308BD0-0CA6-4CE0-9A50-FF6973CEF1CA}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="33" t="s">
+        <v>88</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="35" t="s">
+        <v>91</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="35" t="s">
+        <v>130</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="G8" s="17" t="s">
+        <v>123</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="G9" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="K9" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="L10" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="41"/>
+      <c r="L11" s="20"/>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="38"/>
+      <c r="L12" s="27"/>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="38"/>
+      <c r="L13" s="27"/>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="38"/>
+      <c r="L14" s="27"/>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="38"/>
+      <c r="L15" s="27"/>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="32"/>
+      <c r="H16" s="20"/>
+      <c r="K16" s="38"/>
+      <c r="L16" s="27"/>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="28"/>
+      <c r="H17" s="27"/>
+      <c r="K17" s="39"/>
+      <c r="L17" s="27"/>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="29"/>
+      <c r="H18" s="27"/>
+      <c r="K18" s="40"/>
+      <c r="L18" s="27"/>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="30"/>
+      <c r="H19" s="27"/>
+      <c r="K19" s="40"/>
+      <c r="L19" s="27"/>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="29"/>
+      <c r="H20" s="27"/>
+      <c r="K20" s="40"/>
+      <c r="L20" s="27"/>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="31"/>
+      <c r="H21" s="27"/>
+      <c r="K21" s="40"/>
+      <c r="L21" s="27"/>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="31"/>
+      <c r="H22" s="27"/>
+      <c r="K22" s="28"/>
+      <c r="L22" s="27"/>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="31"/>
+      <c r="H23" s="27"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="27"/>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F78F5A24-06D9-4613-ADF6-9B740818E26F}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="59" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="34" t="s">
+        <v>138</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="34" t="s">
+        <v>139</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="59" t="s">
+        <v>90</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="42" t="s">
+        <v>135</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G16" s="43" t="s">
+        <v>136</v>
+      </c>
+      <c r="H16" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="32"/>
+      <c r="H17" s="20"/>
+      <c r="K17" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G18" s="29"/>
+      <c r="H18" s="27"/>
+      <c r="K18" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="L18" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="30"/>
+      <c r="H19" s="27"/>
+      <c r="K19" s="45"/>
+      <c r="L19" s="20"/>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="29"/>
+      <c r="H20" s="27"/>
+      <c r="K20" s="44"/>
+      <c r="L20" s="27"/>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="31"/>
+      <c r="H21" s="27"/>
+      <c r="K21" s="44"/>
+      <c r="L21" s="27"/>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="31"/>
+      <c r="H22" s="27"/>
+      <c r="K22" s="44"/>
+      <c r="L22" s="27"/>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="31"/>
+      <c r="H23" s="27"/>
+      <c r="K23" s="44"/>
+      <c r="L23" s="27"/>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F66EF12-2E01-4796-A04D-3CC5263B96D7}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="47" t="s">
+        <v>132</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="50" t="s">
+        <v>138</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="68" t="s">
+        <v>163</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="47" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="34" t="s">
+        <v>140</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="59" t="s">
+        <v>143</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="59" t="s">
+        <v>144</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="34" t="s">
+        <v>137</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="34" t="s">
+        <v>164</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K17" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G18" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K18" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="G19" s="22" t="s">
+        <v>194</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="L19" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="43" t="s">
+        <v>147</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K22" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K23" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="61" t="s">
+        <v>148</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K24" s="16" t="s">
+        <v>93</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="61" t="s">
+        <v>149</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="L25" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="62" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="K27" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="L27" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="62" t="s">
+        <v>151</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+    </row>
+    <row r="29" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G29" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G30" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+    </row>
+    <row r="31" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G31" s="62" t="s">
+        <v>154</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G32" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="H32" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="63" t="s">
+        <v>156</v>
+      </c>
+      <c r="H33" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H34" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="25" t="s">
+        <v>157</v>
+      </c>
+      <c r="H35" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G36" s="25" t="s">
+        <v>158</v>
+      </c>
+      <c r="H36" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="H37" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{092F5795-A134-4210-B2B0-D916144240D9}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="46" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="51" t="s">
+        <v>130</v>
+      </c>
+      <c r="L3" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="L4" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="L6" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="L7" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="58" t="s">
+        <v>166</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="L8" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>104</v>
+      </c>
+      <c r="L9" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>95</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="L11" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="L12" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="L13" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="59" t="s">
+        <v>167</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="L17" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="L18" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G19" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="L19" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="L20" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="L21" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="L22" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="L23" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G24" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="L24" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K25" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="L25" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="K26" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="L26" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="K27" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="L27" s="19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="K29" s="27"/>
+      <c r="L29" s="27"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="K30" s="27"/>
+      <c r="L30" s="27"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06F03CB9-C806-4868-9E11-49F2A0DE8B6D}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="52" t="s">
+        <v>138</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="52" t="s">
+        <v>132</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>162</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="52" t="s">
+        <v>109</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="52" t="s">
+        <v>117</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="64" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="52" t="s">
+        <v>101</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G7" s="52" t="s">
+        <v>177</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="52" t="s">
+        <v>100</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="52" t="s">
+        <v>157</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G9" s="52" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="52" t="s">
+        <v>139</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G10" s="52" t="s">
+        <v>159</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="52" t="s">
+        <v>118</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="52" t="s">
+        <v>195</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="52" t="s">
+        <v>99</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G12" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="L12" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G13" s="53" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="52" t="s">
+        <v>95</v>
+      </c>
+      <c r="L13" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G14" s="53" t="s">
+        <v>145</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="L14" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G15" s="53" t="s">
+        <v>103</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="52" t="s">
+        <v>88</v>
+      </c>
+      <c r="L15" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G16" s="66" t="s">
+        <v>178</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="64" t="s">
+        <v>184</v>
+      </c>
+      <c r="L16" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G17" s="66" t="s">
+        <v>179</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K17" s="52" t="s">
+        <v>164</v>
+      </c>
+      <c r="L17" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="66" t="s">
+        <v>180</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K18" s="53" t="s">
+        <v>114</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G19" s="66" t="s">
+        <v>181</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K19" s="53" t="s">
+        <v>116</v>
+      </c>
+      <c r="L19" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G20" s="51" t="s">
+        <v>182</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K20" s="66" t="s">
+        <v>185</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="54" t="s">
+        <v>107</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K21" s="53" t="s">
+        <v>97</v>
+      </c>
+      <c r="L21" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G22" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K22" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="L22" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G23" s="65" t="s">
+        <v>183</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K23" s="51" t="s">
+        <v>186</v>
+      </c>
+      <c r="L23" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G24" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K24" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="K25" s="69" t="s">
+        <v>187</v>
+      </c>
+      <c r="L25" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="K26" s="69" t="s">
+        <v>188</v>
+      </c>
+      <c r="L26" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="K27" s="69" t="s">
+        <v>189</v>
+      </c>
+      <c r="L27" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72983E84-249F-406E-9E63-A9ACF895D43B}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="H3" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K3" s="55" t="s">
+        <v>118</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G4" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K4" s="55" t="s">
+        <v>186</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G5" s="55" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="55" t="s">
+        <v>117</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G6" s="55" t="s">
+        <v>177</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K6" s="55" t="s">
+        <v>138</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G7" s="67" t="s">
+        <v>190</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K7" s="55" t="s">
+        <v>162</v>
+      </c>
+      <c r="L7" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="55" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K8" s="55" t="s">
+        <v>91</v>
+      </c>
+      <c r="L8" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G9" s="55" t="s">
+        <v>147</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K9" s="55" t="s">
+        <v>102</v>
+      </c>
+      <c r="L9" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G10" s="55" t="s">
+        <v>107</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K10" s="55" t="s">
+        <v>100</v>
+      </c>
+      <c r="L10" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="55" t="s">
+        <v>98</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K11" s="55" t="s">
+        <v>99</v>
+      </c>
+      <c r="L11" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G12" s="55" t="s">
+        <v>132</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K12" s="55" t="s">
+        <v>106</v>
+      </c>
+      <c r="L12" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G13" s="67" t="s">
+        <v>191</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K13" s="55" t="s">
+        <v>114</v>
+      </c>
+      <c r="L13" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G14" s="55" t="s">
+        <v>182</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K14" s="55" t="s">
+        <v>116</v>
+      </c>
+      <c r="L14" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G15" s="55" t="s">
+        <v>134</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K15" s="55" t="s">
+        <v>101</v>
+      </c>
+      <c r="L15" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G16" s="67" t="s">
+        <v>192</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="K16" s="55" t="s">
+        <v>164</v>
+      </c>
+      <c r="L16" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="K17" s="55" t="s">
+        <v>139</v>
+      </c>
+      <c r="L17" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="K18" s="67" t="s">
+        <v>104</v>
+      </c>
+      <c r="L18" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="K19" s="55" t="s">
+        <v>137</v>
+      </c>
+      <c r="L19" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="K20" s="55" t="s">
+        <v>97</v>
+      </c>
+      <c r="L20" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="K21" s="55" t="s">
+        <v>95</v>
+      </c>
+      <c r="L21" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="K22" s="56" t="s">
+        <v>165</v>
+      </c>
+      <c r="L22" s="57" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="21"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="K27" s="21"/>
+      <c r="L27" s="21"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="K29" s="21"/>
+      <c r="L29" s="21"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="K30" s="21"/>
+      <c r="L30" s="21"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="K31" s="21"/>
+      <c r="L31" s="21"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="K34" s="21"/>
+      <c r="L34" s="21"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="K35" s="21"/>
+      <c r="L35" s="21"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="21"/>
+      <c r="H37" s="21"/>
+      <c r="K37" s="21"/>
+      <c r="L37" s="21"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="K38" s="21"/>
+      <c r="L38" s="21"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="K40" s="21"/>
+      <c r="L40" s="21"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="K41" s="21"/>
+      <c r="L41" s="21"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="K42" s="21"/>
+      <c r="L42" s="21"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>